<commit_message>
Carpetas con Evidencias, Logs y Reportes
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01E366F1-86B6-4B2D-BB54-9D7691EB8ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="11835" activeTab="2"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
   <si>
     <t>Key</t>
   </si>
@@ -41,23 +42,125 @@
     <t>Exceptions_Screenshots</t>
   </si>
   <si>
+    <t>DummyShouldStopMasterAssetName</t>
+  </si>
+  <si>
+    <t>ShouldStopMasterAssetName</t>
+  </si>
+  <si>
+    <t>https://fakestoreapi.com/products</t>
+  </si>
+  <si>
     <t>QueueName</t>
   </si>
   <si>
+    <t>ProviderName</t>
+  </si>
+  <si>
+    <t>UrlFakeStoreApi</t>
+  </si>
+  <si>
+    <t>URL Fake Store API</t>
+  </si>
+  <si>
+    <t>PathReports</t>
+  </si>
+  <si>
+    <t>UrlOneDrive</t>
+  </si>
+  <si>
+    <t>Client ID de Microsoft Entra</t>
+  </si>
+  <si>
+    <t>ClientId App GraphAPI</t>
+  </si>
+  <si>
+    <t>Valor de Client Secret App GraphAPI</t>
+  </si>
+  <si>
+    <t>Ruta reportes Excel</t>
+  </si>
+  <si>
     <t>TestQueue</t>
   </si>
   <si>
-    <t>DummyShouldStopMasterAssetName</t>
-  </si>
-  <si>
-    <t>ShouldStopMasterAssetName</t>
+    <t>Ruta archivos json OneDrive</t>
+  </si>
+  <si>
+    <t>AZ_TENANT_ID</t>
+  </si>
+  <si>
+    <t>AZ_CLIENT_ID</t>
+  </si>
+  <si>
+    <t>AZ_CLIENT_SECRET</t>
+  </si>
+  <si>
+    <t>https://graph.microsoft.com/v1.0/users/Ronald921704@hotmail.com/drive/RPA/</t>
+  </si>
+  <si>
+    <t>C:\Users\Ronal\AppData\Local\PIX\Projects\OPS_001_AnalisisProductos\Logs</t>
+  </si>
+  <si>
+    <t>C:\Users\Ronal\AppData\Local\PIX\Projects\OPS_001_AnalisisProductos\Evidencias</t>
+  </si>
+  <si>
+    <t>C:\Users\Ronal\AppData\Local\PIX\Projects\OPS_001_AnalisisProductos\Reportes</t>
+  </si>
+  <si>
+    <t>PathLogs</t>
+  </si>
+  <si>
+    <t>CollaboratorName</t>
+  </si>
+  <si>
+    <t>Nombre Colaborador Google Form</t>
+  </si>
+  <si>
+    <t>Ronald Guarín</t>
+  </si>
+  <si>
+    <t>ConnString</t>
+  </si>
+  <si>
+    <t>System.Data.Odbc</t>
+  </si>
+  <si>
+    <t>Driver={ODBC Driver 18 for SQL Server};Server=ASUSVivoAIO\SQLEXPRESS;Database=Productos;Trusted_Connection=Yes;TrustServerCertificate=Yes;</t>
+  </si>
+  <si>
+    <t>PathEvidences</t>
+  </si>
+  <si>
+    <t>URL Google Form carga de Archivos</t>
+  </si>
+  <si>
+    <t>Proveedor Conexión SQL</t>
+  </si>
+  <si>
+    <t>Cadena de conexión a SQL Server</t>
+  </si>
+  <si>
+    <t>UrlGoogleForm</t>
+  </si>
+  <si>
+    <t>https://forms.gle/73JRFo2tBfiYiPC2A</t>
+  </si>
+  <si>
+    <t>Ruta para guardar archivos json</t>
+  </si>
+  <si>
+    <t>Ruta evidencias envío de formulario</t>
+  </si>
+  <si>
+    <t>Cola para gestión de procesos</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -72,6 +175,28 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -92,14 +217,23 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -377,16 +511,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.5703125" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="26.7109375" customWidth="1"/>
+    <col min="2" max="2" width="135.28515625" customWidth="1"/>
+    <col min="3" max="3" width="47.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -397,23 +531,156 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{2749B92B-72F9-476C-B5E3-979156BE1496}"/>
+    <hyperlink ref="B13" r:id="rId2" xr:uid="{C081E99C-2900-4C06-848C-838D88251EF6}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{E2AB3C35-21DA-458A-B157-1B2D8FB58F6D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9C65160-A8E0-446E-AF4F-971CC91598A3}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.85546875" customWidth="1"/>
     <col min="2" max="2" width="35.140625" bestFit="1" customWidth="1"/>
@@ -436,7 +703,7 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -449,10 +716,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -462,9 +729,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36020AE9-9DBE-489C-A1AC-B86CE2043714}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:3" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">

</xml_diff>